<commit_message>
feat(wts): ship B+E revenue OS, A affiliate face; park C+D
Implement Docs B+E as the operating system (scoped Footprint/Growth/
Automation retainers, commissions/tiers) and Doc A Regional Hustler
messaging on affiliate-sales. Prices page hard caps + Laos/Thailand notes.
Park C (directory) + D (cards) as future platform feeds only.
Also clean fr/la/th redirect stubs after merge conflict markers.
</commit_message>
<xml_diff>
--- a/docs/WTS-Product-Menu-from-Legacy-Deck.xlsx
+++ b/docs/WTS-Product-Menu-from-Legacy-Deck.xlsx
@@ -963,9 +963,6 @@
           <t>$50/m</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -1028,7 +1025,6 @@
           <t>$26</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -2091,8 +2087,6 @@
           <t>$800</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -2150,8 +2144,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -2502,7 +2494,6 @@
           <t>OOH/media network outside WTS positioning</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2565,7 +2556,6 @@
           <t>OOH/media network outside WTS positioning</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2603,8 +2593,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -2620,7 +2608,6 @@
           <t>OOH/media network outside WTS positioning</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2658,8 +2645,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -2675,7 +2660,6 @@
           <t>OOH/media network outside WTS positioning</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2713,8 +2697,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -2730,7 +2712,6 @@
           <t>OOH/media network outside WTS positioning</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2768,8 +2749,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -2785,7 +2764,6 @@
           <t>OOH/media network outside WTS positioning</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2823,8 +2801,6 @@
           <t>$0.95</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -3959,7 +3935,6 @@
           <t>$65</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
           <t>1 time</t>
@@ -4211,7 +4186,6 @@
           <t>False</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>COWE01 adapted for SEA SME pricing</t>
@@ -4279,7 +4253,6 @@
           <t>False</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>COWE02</t>
@@ -4419,7 +4392,6 @@
           <t>False</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>COWE04/05/07</t>
@@ -4487,7 +4459,6 @@
           <t>False</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>Legacy copy + glossary engine</t>
@@ -4555,7 +4526,6 @@
           <t>False</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>COLM lead magnets</t>
@@ -4623,7 +4593,6 @@
           <t>False</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>Social SKUs + Digital Footprint</t>
@@ -4713,7 +4682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4824,6 +4793,114 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OS rule</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B+E=revenue OS; A=affiliate face; C+D=future platforms only</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Package rule</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Scoped retainers with hard caps — not unlimited catalogue delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Doc A</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1HvQCCq_PMSBo7SYk-0-h5ixDw0zmhaSsZ-IGC93dHC0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Doc B</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1khzaiupSabNEQqNFG4xK8I4gNrqH5MG60X2qXcVetgw</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Doc C (parked)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1qRygOFE16GSqhYKP8Z6GwFzVnRpJAkXStZUHafyNjPs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Doc D (parked)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1M5ohlm4RHpbEJATEw_RHV-2RT4LbdMvPhei2QFkcVzs</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Doc E</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1SQH_TQKQ51UnQejp1gwgp1Gss9WT4oZFhHolIuoFOa8</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>OS markdown</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>docs/WTS-Revenue-Affiliate-OS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Updated OS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(wts): map Doc F NLHS strategy as Laos flywheel into revenue OS
National Lao Home Show internal strategy feeds vendor digitization and
recurring retainers; does not replace B+E product/affiliate OS or A face.
Confidential framing stays off public site.
</commit_message>
<xml_diff>
--- a/docs/WTS-Product-Menu-from-Legacy-Deck.xlsx
+++ b/docs/WTS-Product-Menu-from-Legacy-Deck.xlsx
@@ -4682,7 +4682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4901,6 +4901,30 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Doc F (NLHS flywheel)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1HwZFql9KXHw1ChD2OnnDwxYa2vEAgJSzzjsWRDI8A5Y — expo feeds WTS retainers; public narrative only on site</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>OS rule update</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>B+E=revenue OS; A=face; F=NLHS GTM flywheel; C+D=future only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>